<commit_message>
Had to fixed gpt-5 Python outputs for meeting, trip, and zebralogic due to parsing issues.
</commit_message>
<xml_diff>
--- a/output/Python/gpt-5-2025-08-07/task_analysis_results_singlepass_Python_gpt-5-2025-08-07_trip.xlsx
+++ b/output/Python/gpt-5-2025-08-07/task_analysis_results_singlepass_Python_gpt-5-2025-08-07_trip.xlsx
@@ -1452,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1502,26 +1502,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_trip()
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Riga"}, {"day_range": "Day 2-7", "place": "Istanbul"}, {"day_range": "Day 7-13", "place": "Krakow"}, {"day_range": "Day 13-15", "place": "Warsaw"}, {"day_range": "Day 15-21", "place": "Reykjavik"}]}</t>
         </is>
       </c>
     </row>
@@ -1535,26 +1531,22 @@
         <v>1</v>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Prague"}, {"day_range": "Day 2-5", "place": "Helsinki"}, {"day_range": "Day 5-8", "place": "Naples"}, {"day_range": "Day 8-10", "place": "Frankfurt"}, {"day_range": "Day 10-12", "place": "Lyon"}]}</t>
         </is>
       </c>
     </row>
@@ -1568,26 +1560,22 @@
         <v>1</v>
       </c>
       <c r="C4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Reykjavik"}, {"day_range": "Day 4-7", "place": "Stuttgart"}, {"day_range": "Day 7-11", "place": "Valencia"}, {"day_range": "Day 11-13", "place": "Seville"}, {"day_range": "Day 13-15", "place": "Munich"}, {"day_range": "Day 15-19", "place": "Geneva"}, {"day_range": "Day 19-22", "place": "Istanbul"}, {"day_range": "Day 22-25", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
@@ -1601,26 +1589,22 @@
         <v>1</v>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "London"}, {"day_range": "Day 2-3", "place": "Madrid"}, {"day_range": "Day 3-7", "place": "Berlin"}, {"day_range": "Day 7-9", "place": "Dublin"}, {"day_range": "Day 9-11", "place": "Oslo"}, {"day_range": "Day 11-13", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
@@ -1634,26 +1618,22 @@
         <v>1</v>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_trip()
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Vilnius"}, {"day_range": "Day 3-7", "place": "Frankfurt"}, {"day_range": "Day 7-9", "place": "Stuttgart"}, {"day_range": "Day 9-10", "place": "London"}, {"day_range": "Day 10-11", "place": "Santorini"}, {"day_range": "Day 11-13", "place": "Dublin"}, {"day_range": "Day 13-17", "place": "Seville"}]}</t>
         </is>
       </c>
     </row>
@@ -1667,26 +1647,22 @@
         <v>1</v>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Vienna"}, {"day_range": "Day 4-6", "place": "Rome"}, {"day_range": "Day 6-7", "place": "Riga"}, {"day_range": "Day 7-10", "place": "Vilnius"}, {"day_range": "Day 10-11", "place": "Milan"}, {"day_range": "Day 11-13", "place": "Lisbon"}, {"day_range": "Day 13-15", "place": "Oslo"}]}</t>
         </is>
       </c>
     </row>
@@ -1700,26 +1676,22 @@
         <v>1</v>
       </c>
       <c r="C8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Helsinki"}, {"day_range": "Day 2-5", "place": "Madrid"}, {"day_range": "Day 5-8", "place": "Budapest"}, {"day_range": "Day 8-9", "place": "Reykjavik"}, {"day_range": "Day 9-11", "place": "Warsaw"}, {"day_range": "Day 11-14", "place": "Split"}]}</t>
         </is>
       </c>
     </row>
@@ -1733,26 +1705,22 @@
         <v>1</v>
       </c>
       <c r="C9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Hamburg"}, {"day_range": "Day 2-4", "place": "Budapest"}, {"day_range": "Day 4-9", "place": "Mykonos"}]}</t>
         </is>
       </c>
     </row>
@@ -1766,26 +1734,22 @@
         <v>1</v>
       </c>
       <c r="C10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Edinburgh"}, {"day_range": "Day 5-8", "place": "Amsterdam"}, {"day_range": "Day 8-12", "place": "Vienna"}, {"day_range": "Day 12-16", "place": "Reykjavik"}, {"day_range": "Day 16-19", "place": "Berlin"}, {"day_range": "Day 19-23", "place": "Brussels"}]}</t>
         </is>
       </c>
     </row>
@@ -1799,26 +1763,22 @@
         <v>1</v>
       </c>
       <c r="C11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Vienna"}, {"day_range": "Day 7-9", "place": "Lyon"}, {"day_range": "Day 9-11", "place": "Amsterdam"}, {"day_range": "Day 11-14", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
@@ -1832,25 +1792,22 @@
         <v>1</v>
       </c>
       <c r="C12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 1
-    Given an order of cities and desired days per city, compute overlapping day ranges.
-          ^^
-SyntaxError: invalid syntax</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Krakow"}, {"day_range": "Day 2-3", "place": "Stuttgart"}, {"day_range": "Day 3-4", "place": "Split"}, {"day_range": "Day 4-7", "place": "Prague"}, {"day_range": "Day 7-8", "place": "Florence"}]}</t>
         </is>
       </c>
     </row>
@@ -1864,26 +1821,22 @@
         <v>1</v>
       </c>
       <c r="C13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "London"}, {"day_range": "Day 7-11", "place": "Split"}, {"day_range": "Day 11-12", "place": "Oslo"}, {"day_range": "Day 12-16", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
@@ -1897,26 +1850,22 @@
         <v>1</v>
       </c>
       <c r="C14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Vilnius"}, {"day_range": "Day 3-7", "place": "Munich"}, {"day_range": "Day 7-11", "place": "Budapest"}, {"day_range": "Day 11-15", "place": "Paris"}, {"day_range": "Day 15-18", "place": "Split"}, {"day_range": "Day 18-22", "place": "Krakow"}, {"day_range": "Day 22-25", "place": "Amsterdam"}, {"day_range": "Day 25-29", "place": "Santorini"}, {"day_range": "Day 29-30", "place": "Geneva"}]}</t>
         </is>
       </c>
     </row>
@@ -1930,26 +1879,22 @@
         <v>1</v>
       </c>
       <c r="C15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Nice"}, {"day_range": "Day 5-8", "place": "Lyon"}, {"day_range": "Day 8-14", "place": "Dublin"}, {"day_range": "Day 14-19", "place": "Krakow"}, {"day_range": "Day 19-20", "place": "Frankfurt"}]}</t>
         </is>
       </c>
     </row>
@@ -1963,26 +1908,22 @@
         <v>1</v>
       </c>
       <c r="C16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Vienna"}, {"day_range": "Day 2-3", "place": "Nice"}, {"day_range": "Day 3-7", "place": "Stockholm"}, {"day_range": "Day 7-9", "place": "Split"}]}</t>
         </is>
       </c>
     </row>
@@ -1996,26 +1937,22 @@
         <v>1</v>
       </c>
       <c r="C17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 16, in &lt;module&gt;
-    result = find_itinerary(total_days, city_stays, direct_flights)
-             ^^^^^^^^^^^^^^
-NameError: name 'find_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Dublin"}, {"day_range": "Day 2-6", "place": "Riga"}, {"day_range": "Day 6-12", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
@@ -2029,26 +1966,22 @@
         <v>1</v>
       </c>
       <c r="C18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "London"}, {"day_range": "Day 3-7", "place": "Milan"}, {"day_range": "Day 7-8", "place": "Zurich"}, {"day_range": "Day 8-9", "place": "Stockholm"}, {"day_range": "Day 9-13", "place": "Reykjavik"}, {"day_range": "Day 13-17", "place": "Stuttgart"}, {"day_range": "Day 17-21", "place": "Hamburg"}, {"day_range": "Day 21-22", "place": "Bucharest"}, {"day_range": "Day 22-25", "place": "Barcelona"}, {"day_range": "Day 25-28", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
@@ -2062,26 +1995,22 @@
         <v>1</v>
       </c>
       <c r="C19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Florence"}, {"day_range": "Day 5-8", "place": "Prague"}, {"day_range": "Day 8-12", "place": "Tallinn"}, {"day_range": "Day 12-16", "place": "Frankfurt"}, {"day_range": "Day 16-18", "place": "Bucharest"}, {"day_range": "Day 18-22", "place": "Zurich"}, {"day_range": "Day 22-26", "place": "Venice"}]}</t>
         </is>
       </c>
     </row>
@@ -2124,26 +2053,22 @@
         <v>1</v>
       </c>
       <c r="C21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Nice"}, {"day_range": "Day 3-4", "place": "Reykjavik"}, {"day_range": "Day 4-5", "place": "Stockholm"}, {"day_range": "Day 5-7", "place": "Split"}, {"day_range": "Day 7-8", "place": "Copenhagen"}, {"day_range": "Day 8-11", "place": "Venice"}, {"day_range": "Day 11-13", "place": "Vienna"}, {"day_range": "Day 13-17", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
@@ -2186,26 +2111,22 @@
         <v>1</v>
       </c>
       <c r="C23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    plan_trip()
-    ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Manchester"}, {"day_range": "Day 7-10", "place": "Madrid"}, {"day_range": "Day 10-11", "place": "Vienna"}, {"day_range": "Day 11-15", "place": "Stuttgart"}]}</t>
         </is>
       </c>
     </row>
@@ -2219,26 +2140,22 @@
         <v>1</v>
       </c>
       <c r="C24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    build_itinerary()
-    ^^^^^^^^^^^^^^^
-NameError: name 'build_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Lyon"}, {"day_range": "Day 4-8", "place": "Paris"}, {"day_range": "Day 8-12", "place": "Copenhagen"}, {"day_range": "Day 12-13", "place": "Santorini"}, {"day_range": "Day 13-17", "place": "Oslo"}, {"day_range": "Day 17-18", "place": "Krakow"}, {"day_range": "Day 18-22", "place": "Helsinki"}, {"day_range": "Day 22-23", "place": "Warsaw"}, {"day_range": "Day 23-24", "place": "Riga"}, {"day_range": "Day 24-25", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
@@ -2252,26 +2169,22 @@
         <v>1</v>
       </c>
       <c r="C25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Hamburg"}, {"day_range": "Day 7-13", "place": "Split"}, {"day_range": "Day 13-14", "place": "Lyon"}, {"day_range": "Day 14-19", "place": "Munich"}, {"day_range": "Day 19-20", "place": "Manchester"}]}</t>
         </is>
       </c>
     </row>
@@ -2285,26 +2198,22 @@
         <v>1</v>
       </c>
       <c r="C26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_trip()
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-6", "place": "Split"}, {"day_range": "Day 6-12", "place": "London"}, {"day_range": "Day 12-18", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
@@ -2318,11 +2227,11 @@
         <v>1</v>
       </c>
       <c r="C27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -2333,11 +2242,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Bucharest"}, {"day_range": "Day 6", "place": "Bucharest -&gt; Warsaw (travel day)"}, {"day_range": "Day 7", "place": "Warsaw -&gt; Stuttgart (travel day)"}, {"day_range": "Day 8-12", "place": "Stuttgart"}, {"day_range": "Day 13", "place": "Stuttgart -&gt; Copenhagen (travel day)"}, {"day_range": "Day 14", "place": "Copenhagen"}, {"day_range": "Day 15", "place": "Copenhagen -&gt; Dubrovnik (travel day)"}, {"day_range": "Day 16-19", "place": "Dubrovnik"}]}</t>
         </is>
       </c>
     </row>
@@ -2351,176 +2256,156 @@
         <v>1</v>
       </c>
       <c r="C28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Santorini"}, {"day_range": "Day 3-6", "place": "Vienna"}, {"day_range": "Day 6-7", "place": "Madrid"}, {"day_range": "Day 7-8", "place": "Seville"}, {"day_range": "Day 8-11", "place": "Valencia"}, {"day_range": "Day 11-15", "place": "Krakow"}, {"day_range": "Day 15-18", "place": "Frankfurt"}, {"day_range": "Day 18-20", "place": "Bucharest"}, {"day_range": "Day 20-23", "place": "Riga"}, {"day_range": "Day 23-27", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>trip_planning_example_1543</t>
+          <t>trip_planning_example_950</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>1</v>
       </c>
       <c r="C29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Rome"}, {"day_range": "Day 4-6", "place": "Mykonos"}, {"day_range": "Day 6-8", "place": "Nice"}, {"day_range": "Day 8-10", "place": "Riga"}, {"day_range": "Day 10-13", "place": "Bucharest"}, {"day_range": "Day 13-16", "place": "Munich"}, {"day_range": "Day 16-17", "place": "Krakow"}]}</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>trip_planning_example_1572</t>
+          <t>trip_planning_example_1543</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_itinerary()
-             ^^^^^^^^^^^^^^
-NameError: name 'plan_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Prague"}, {"day_range": "Day 3-5", "place": "London"}, {"day_range": "Day 5-9", "place": "Lisbon"}, {"day_range": "Day 9-11", "place": "Athens"}, {"day_range": "Day 11-13", "place": "Dubrovnik"}, {"day_range": "Day 13-15", "place": "Dublin"}, {"day_range": "Day 15-16", "place": "Seville"}, {"day_range": "Day 16-20", "place": "Porto"}, {"day_range": "Day 20-23", "place": "Warsaw"}, {"day_range": "Day 23-26", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>trip_planning_example_1596</t>
+          <t>trip_planning_example_1572</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>1</v>
       </c>
       <c r="C31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Berlin"}, {"day_range": "Day 2-4", "place": "Milan"}, {"day_range": "Day 4-6", "place": "Seville"}, {"day_range": "Day 6-10", "place": "Paris"}, {"day_range": "Day 10-12", "place": "Lyon"}, {"day_range": "Day 12-13", "place": "Nice"}, {"day_range": "Day 13-16", "place": "Naples"}, {"day_range": "Day 16-20", "place": "Zurich"}, {"day_range": "Day 20-22", "place": "Stockholm"}, {"day_range": "Day 22-23", "place": "Riga"}]}</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>trip_planning_example_857</t>
+          <t>trip_planning_example_1596</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>1</v>
       </c>
       <c r="C32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Edinburgh"}, {"day_range": "Day 5-9", "place": "Barcelona"}, {"day_range": "Day 9-13", "place": "Budapest"}, {"day_range": "Day 13-17", "place": "Vienna"}, {"day_range": "Day 17-18", "place": "Stockholm"}, {"day_range": "Day 18-20", "place": "Munich"}, {"day_range": "Day 20-21", "place": "Bucharest"}, {"day_range": "Day 21-25", "place": "Riga"}, {"day_range": "Day 25-29", "place": "Warsaw"}, {"day_range": "Day 29-32", "place": "Krakow"}]}</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>trip_planning_example_344</t>
+          <t>trip_planning_example_857</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>1</v>
       </c>
       <c r="C33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -2531,183 +2416,159 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = solve_itinerary()
-             ^^^^^^^^^^^^^^^
-NameError: name 'solve_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Porto"}, {"day_range": "Day 3-7", "place": "Hamburg"}, {"day_range": "Day 5-6", "place": "Frankfurt"}, {"day_range": "Day 7-9", "place": "Geneva"}, {"day_range": "Day 9-11", "place": "Mykonos"}, {"day_range": "Day 11-15", "place": "Naples"}, {"day_range": "Day 15-18", "place": "Manchester"}]}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>trip_planning_example_90</t>
+          <t>trip_planning_example_344</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = build_itinerary()
-             ^^^^^^^^^^^^^^^
-NameError: name 'build_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-6", "place": "Athens"}, {"day_range": "Day 6-11", "place": "Zurich"}, {"day_range": "Day 11-16", "place": "Valencia"}, {"day_range": "Day 16-20", "place": "Naples"}]}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>trip_planning_example_699</t>
+          <t>trip_planning_example_90</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = build_itinerary()
-             ^^^^^^^^^^^^^^^
-NameError: name 'build_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Naples"}, {"day_range": "Day 5-11", "place": "Vienna"}, {"day_range": "Day 11-17", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>trip_planning_example_934</t>
+          <t>trip_planning_example_699</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Hamburg"}, {"day_range": "Day 2-6", "place": "Dublin"}, {"day_range": "Day 6-9", "place": "Helsinki"}, {"day_range": "Day 9-10", "place": "Reykjavik"}, {"day_range": "Day 10-14", "place": "London"}, {"day_range": "Day 14-16", "place": "Mykonos"}]}</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>trip_planning_example_275</t>
+          <t>trip_planning_example_934</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Dubrovnik"}, {"day_range": "Day 3-4", "place": "Rome"}, {"day_range": "Day 4-7", "place": "Riga"}, {"day_range": "Day 7-11", "place": "Brussels"}, {"day_range": "Day 11-12", "place": "Valencia"}, {"day_range": "Day 12-16", "place": "Geneva"}, {"day_range": "Day 16-17", "place": "Budapest"}]}</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>trip_planning_example_675</t>
+          <t>trip_planning_example_275</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Vilnius"}, {"day_range": "Day 4-8", "place": "Split"}, {"day_range": "Day 8-13", "place": "Madrid"}, {"day_range": "Day 13-14", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>trip_planning_example_1075</t>
+          <t>trip_planning_example_675</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2730,28 +2591,29 @@
       <c r="G39" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 115, in &lt;module&gt;
     main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 77, in main
+    for c, days in city_days.items:
+TypeError: 'builtin_function_or_method' object is not iterable</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>trip_planning_example_409</t>
+          <t>trip_planning_example_1075</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E40" t="b">
@@ -2762,29 +2624,25 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Manchester"}, {"day_range": "Day 2-5", "place": "Prague"}, {"day_range": "Day 5-8", "place": "Edinburgh"}, {"day_range": "Day 8-12", "place": "Stuttgart"}, {"day_range": "Day 12-16", "place": "Reykjavik"}, {"day_range": "Day 16-19", "place": "Vienna"}, {"day_range": "Day 19-23", "place": "Split"}, {"day_range": "Day 23-25", "place": "Lyon"}]}</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>trip_planning_example_1534</t>
+          <t>trip_planning_example_409</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>1</v>
       </c>
       <c r="C41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E41" t="b">
@@ -2795,18 +2653,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Zurich"}, {"day_range": "Day 3", "place": "Zurich -&gt; Helsinki (flight day)"}, {"day_range": "Day 4", "place": "Helsinki -&gt; Split (flight day)"}, {"day_range": "Day 5-9", "place": "Split"}, {"day_range": "Day 10", "place": "Split -&gt; Hamburg (flight day)"}, {"day_range": "Day 11", "place": "Hamburg -&gt; Bucharest (flight day)"}, {"day_range": "Day 12", "place": "Bucharest"}]}</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>trip_planning_example_1559</t>
+          <t>trip_planning_example_1534</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2829,149 +2683,134 @@
       <c r="G42" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 218, in &lt;module&gt;
     main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 152, in main
+    raise ValueError(f"City {city} has {city_counts.get(city, 0)} days, required {req_days}")
+ValueError: City Tallinn has 3 days, required 2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>trip_planning_example_113</t>
+          <t>trip_planning_example_1559</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>1</v>
       </c>
       <c r="C43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Prague"}, {"day_range": "Day 3-4", "place": "Valencia"}, {"day_range": "Day 4-5", "place": "Lisbon"}, {"day_range": "Day 5-9", "place": "Seville"}, {"day_range": "Day 9-12", "place": "Paris"}, {"day_range": "Day 12-13", "place": "Tallinn"}, {"day_range": "Day 13-15", "place": "Oslo"}, {"day_range": "Day 15-18", "place": "Lyon"}, {"day_range": "Day 18-21", "place": "Nice"}, {"day_range": "Day 21-25", "place": "Mykonos"}]}</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>trip_planning_example_149</t>
+          <t>trip_planning_example_113</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>1</v>
       </c>
       <c r="C44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Naples"}, {"day_range": "Day 3-9", "place": "Milan"}, {"day_range": "Day 9-12", "place": "Seville"}]}</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>trip_planning_example_1088</t>
+          <t>trip_planning_example_149</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>1</v>
       </c>
       <c r="C45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Istanbul"}, {"day_range": "Day 3-5", "place": "London"}, {"day_range": "Day 5-10", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>trip_planning_example_1487</t>
+          <t>trip_planning_example_1088</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>1</v>
       </c>
       <c r="C46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Reykjavik"}, {"day_range": "Day 2-4", "place": "Stockholm"}, {"day_range": "Day 4-8", "place": "Tallinn"}, {"day_range": "Day 8-12", "place": "Oslo"}, {"day_range": "Day 12-13", "place": "Geneva"}, {"day_range": "Day 13-15", "place": "Split"}, {"day_range": "Day 15-19", "place": "Stuttgart"}, {"day_range": "Day 19-21", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>trip_planning_example_777</t>
+          <t>trip_planning_example_1487</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2994,61 +2833,58 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 215, in &lt;module&gt;
     main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 202, in main
+    raise RuntimeError("No feasible itinerary found under given constraints.")
+RuntimeError: No feasible itinerary found under given constraints.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>trip_planning_example_657</t>
+          <t>trip_planning_example_777</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>1</v>
       </c>
       <c r="C48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Reykjavik"}, {"day_range": "Day 2-3", "place": "Vienna"}, {"day_range": "Day 3-5", "place": "Helsinki"}, {"day_range": "Day 5-7", "place": "Riga"}, {"day_range": "Day 7-11", "place": "Tallinn"}, {"day_range": "Day 11-15", "place": "Dublin"}]}</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>trip_planning_example_769</t>
+          <t>trip_planning_example_657</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>1</v>
       </c>
       <c r="C49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -3059,62 +2895,54 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1", "place": "Valencia"}, {"day_range": "Day 2", "place": "Valencia"}, {"day_range": "Day 3", "place": "Valencia"}, {"day_range": "Day 4", "place": "Valencia -&gt; Naples (flight day)"}, {"day_range": "Day 5", "place": "Naples"}, {"day_range": "Day 6", "place": "Naples"}, {"day_range": "Day 7", "place": "Naples -&gt; Manchester (flight day)"}, {"day_range": "Day 8", "place": "Manchester"}, {"day_range": "Day 9", "place": "Manchester"}, {"day_range": "Day 10", "place": "Manchester -&gt; Oslo (flight day)"}, {"day_range": "Day 11", "place": "Oslo"}, {"day_range": "Day 12", "place": "Oslo -&gt; Vilnius (flight day)"}, {"day_range": "Day 13", "place": "Vilnius -&gt; Frankfurt (flight day)"}, {"day_range": "Day 14", "place": "Frankfurt"}, {"day_range": "Day 15", "place": "Frankfurt"}, {"day_range": "Day 16", "place": "Frankfurt"}]}</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>trip_planning_example_1480</t>
+          <t>trip_planning_example_769</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>1</v>
       </c>
       <c r="C50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Prague"}, {"day_range": "Day 4-7", "place": "Reykjavik"}, {"day_range": "Day 7-10", "place": "Munich"}, {"day_range": "Day 10-14", "place": "Porto"}, {"day_range": "Day 14-15", "place": "Amsterdam"}, {"day_range": "Day 15-16", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>trip_planning_example_1511</t>
+          <t>trip_planning_example_1480</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>1</v>
       </c>
       <c r="C51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -3125,29 +2953,25 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Geneva"}, {"day_range": "Day 4-7", "place": "Istanbul"}, {"day_range": "Day 7-11", "place": "Venice"}, {"day_range": "Day 11-14", "place": "Madrid"}, {"day_range": "Day 14-18", "place": "Munich"}, {"day_range": "Day 18-19", "place": "Reykjavik"}, {"day_range": "Day 19-22", "place": "Vienna"}, {"day_range": "Day 22-23", "place": "Riga"}, {"day_range": "Day 23-26", "place": "Vilnius"}, {"day_range": "Day 26-27", "place": "Brussels"}]}</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>trip_planning_example_709</t>
+          <t>trip_planning_example_1511</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>1</v>
       </c>
       <c r="C52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E52" t="b">
@@ -3158,62 +2982,54 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day": "Day 1", "places": ["Tallinn"]}, {"day": "Day 2", "places": ["Tallinn"]}, {"day": "Day 3", "places": ["Tallinn"]}, {"day": "Day 4", "places": ["Tallinn", "Munich"]}, {"day": "Day 5", "places": ["Munich"]}, {"day": "Day 6", "places": ["Munich", "Venice"]}, {"day": "Day 7", "places": ["Venice"]}, {"day": "Day 8", "places": ["Venice", "Santorini"]}, {"day": "Day 9", "places": ["Santorini"]}, {"day": "Day 10", "places": ["Santorini", "Manchester"]}, {"day": "Day 11", "places": ["Manchester"]}, {"day": "Day 12", "places": ["Manchester", "Porto"]}, {"day": "Day 13", "places": ["Porto"]}, {"day": "Day 14", "places": ["Porto", "Valencia"]}, {"day": "Day 15", "places": ["Valencia", "Bucharest"]}, {"day": "Day 16", "places": ["Bucharest"]}, {"day": "Day 17", "places": ["Bucharest"]}, {"day": "Day 18", "places": ["Bucharest"]}, {"day": "Day 19", "places": ["Bucharest", "Vienna"]}, {"day": "Day 20", "places": ["Vienna"]}, {"day": "Day 21", "places": ["Vienna"]}, {"day": "Day</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>trip_planning_example_1116</t>
+          <t>trip_planning_example_709</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>1</v>
       </c>
       <c r="C53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Dubrovnik"}, {"day_range": "Day 4-7", "place": "Helsinki"}, {"day_range": "Day 7-10", "place": "Reykjavik"}, {"day_range": "Day 10-12", "place": "Prague"}, {"day_range": "Day 12-16", "place": "Valencia"}, {"day_range": "Day 16-18", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>trip_planning_example_142</t>
+          <t>trip_planning_example_1116</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>1</v>
       </c>
       <c r="C54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -3224,128 +3040,112 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Stockholm"}, {"day_range": "Day 4-6", "place": "Split"}, {"day_range": "Day 6-8", "place": "Barcelona"}, {"day_range": "Day 8-12", "place": "Reykjavik"}, {"day_range": "Day 12-15", "place": "Munich"}, {"day_range": "Day 15-16", "place": "Bucharest"}, {"day_range": "Day 16-17", "place": "Oslo"}, {"day_range": "Day 17-20", "place": "Frankfurt"}]}</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>trip_planning_example_591</t>
+          <t>trip_planning_example_142</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>1</v>
       </c>
       <c r="C55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Madrid"}, {"day_range": "Day 4-6", "place": "Dublin"}, {"day_range": "Day 6-7", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>trip_planning_example_1432</t>
+          <t>trip_planning_example_591</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>1</v>
       </c>
       <c r="C56" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Geneva"}, {"day_range": "Day 4-10", "place": "Munich"}, {"day_range": "Day 10-11", "place": "Bucharest"}, {"day_range": "Day 11-16", "place": "Valencia"}, {"day_range": "Day 16-17", "place": "Stuttgart"}]}</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>trip_planning_example_812</t>
+          <t>trip_planning_example_1432</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>1</v>
       </c>
       <c r="C57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Stockholm"}, {"day_range": "Day 3-5", "place": "Amsterdam"}, {"day_range": "Day 5-6", "place": "Valencia"}, {"day_range": "Day 6-10", "place": "Vienna"}, {"day_range": "Day 10-14", "place": "Reykjavik"}, {"day_range": "Day 14-18", "place": "Athens"}, {"day_range": "Day 18-20", "place": "Riga"}, {"day_range": "Day 20-22", "place": "Bucharest"}, {"day_range": "Day 22-25", "place": "Frankfurt"}, {"day_range": "Day 25-29", "place": "Salzburg"}]}</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>trip_planning_example_126</t>
+          <t>trip_planning_example_812</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>1</v>
       </c>
       <c r="C58" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E58" t="b">
@@ -3356,194 +3156,170 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Porto"}, {"day_range": "Day 3-6", "place": "Paris"}, {"day_range": "Day 7-8", "place": "Florence"}, {"day_range": "Day 9-12", "place": "Munich"}, {"day_range": "Day 13-14", "place": "Warsaw"}, {"day_range": "Day 15-18", "place": "Nice"}, {"day_range": "Day 19-20", "place": "Vienna"}]}</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>trip_planning_example_240</t>
+          <t>trip_planning_example_126</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>1</v>
       </c>
       <c r="C59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Krakow"}, {"day_range": "Day 5-6", "place": "Paris"}, {"day_range": "Day 6-11", "place": "Seville"}]}</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>trip_planning_example_440</t>
+          <t>trip_planning_example_240</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>1</v>
       </c>
       <c r="C60" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Prague"}, {"day_range": "Day 2-6", "place": "Stockholm"}, {"day_range": "Day 6-8", "place": "Berlin"}, {"day_range": "Day 8-12", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>trip_planning_example_1424</t>
+          <t>trip_planning_example_440</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>1</v>
       </c>
       <c r="C61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-6", "place": "Geneva"}, {"day_range": "Day 6-7", "place": "Split"}, {"day_range": "Day 7-9", "place": "Vilnius"}, {"day_range": "Day 9-10", "place": "Helsinki"}, {"day_range": "Day 10-12", "place": "Reykjavik"}]}</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>trip_planning_example_1330</t>
+          <t>trip_planning_example_1424</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>1</v>
       </c>
       <c r="C62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Porto"}, {"day_range": "Day 5-8", "place": "Amsterdam"}, {"day_range": "Day 8-11", "place": "Helsinki"}, {"day_range": "Day 11-15", "place": "Reykjavik"}, {"day_range": "Day 15-17", "place": "Warsaw"}, {"day_range": "Day 17-20", "place": "Naples"}, {"day_range": "Day 20-22", "place": "Brussels"}, {"day_range": "Day 22-23", "place": "Valencia"}, {"day_range": "Day 23-25", "place": "Lyon"}, {"day_range": "Day 25-27", "place": "Split"}]}</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>trip_planning_example_1148</t>
+          <t>trip_planning_example_1330</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>1</v>
       </c>
       <c r="C63" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Salzburg"}, {"day_range": "Day 2-5", "place": "Hamburg"}, {"day_range": "Day 5-9", "place": "Venice"}, {"day_range": "Day 9-11", "place": "Nice"}, {"day_range": "Day 11-15", "place": "Zurich"}, {"day_range": "Day 15-18", "place": "Bucharest"}, {"day_range": "Day 18-21", "place": "Copenhagen"}, {"day_range": "Day 21-22", "place": "Brussels"}, {"day_range": "Day 22-25", "place": "Naples"}]}</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>trip_planning_example_768</t>
+          <t>trip_planning_example_1148</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>1</v>
       </c>
       <c r="C64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E64" t="b">
@@ -3554,18 +3330,14 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-1", "place": "Tallinn"}, {"day_range": "Day 2-3", "place": "Prague"}, {"day_range": "Day 4-4", "place": "Lisbon"}, {"day_range": "Day 5-8", "place": "Copenhagen"}, {"day_range": "Day 9-12", "place": "Dubrovnik"}, {"day_range": "Day 13-15", "place": "Stockholm"}, {"day_range": "Day 16-17", "place": "Split"}, {"day_range": "Day 18-19", "place": "Lyon"}]}</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>trip_planning_example_1318</t>
+          <t>trip_planning_example_768</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -3588,94 +3360,88 @@
       <c r="G65" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 190, in &lt;module&gt;
+    result = plan_trip()
+             ^^^^^^^^^^^
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 165, in plan_trip
+    raise RuntimeError("No feasible itinerary found with given constraints.")
+RuntimeError: No feasible itinerary found with given constraints.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>trip_planning_example_29</t>
+          <t>trip_planning_example_1318</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>1</v>
       </c>
       <c r="C66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    compute_itinerary()
-    ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Edinburgh"}, {"day_range": "Day 3-4", "place": "Riga"}, {"day_range": "Day 4-8", "place": "Tallinn"}, {"day_range": "Day 8-12", "place": "Vilnius"}, {"day_range": "Day 12-13", "place": "Helsinki"}, {"day_range": "Day 13-17", "place": "Budapest"}, {"day_range": "Day 17-20", "place": "Geneva"}, {"day_range": "Day 20-24", "place": "Porto"}, {"day_range": "Day 24-25", "place": "Oslo"}]}</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>trip_planning_example_1009</t>
+          <t>trip_planning_example_29</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>1</v>
       </c>
       <c r="C67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Dubrovnik"}, {"day_range": "Day 7-9", "place": "Frankfurt"}, {"day_range": "Day 9-10", "place": "Krakow"}]}</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>trip_planning_example_59</t>
+          <t>trip_planning_example_1009</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>1</v>
       </c>
       <c r="C68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E68" t="b">
@@ -3686,51 +3452,43 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = find_itinerary()
-             ^^^^^^^^^^^^^^
-NameError: name 'find_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Florence"}, {"day_range": "Day 4-5", "place": "Vienna"}, {"day_range": "Day 5-8", "place": "Reykjavik"}, {"day_range": "Day 8-12", "place": "Stuttgart"}, {"day_range": "Day 12-13", "place": "Istanbul"}, {"day_range": "Day 13-16", "place": "Riga"}, {"day_range": "Day 16-19", "place": "Bucharest"}, {"day_range": "Day 19-23", "place": "Manchester"}]}</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>trip_planning_example_1568</t>
+          <t>trip_planning_example_59</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>1</v>
       </c>
       <c r="C69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Bucharest"}, {"day_range": "Day 7-13", "place": "Lyon"}, {"day_range": "Day 13-16", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>trip_planning_example_339</t>
+          <t>trip_planning_example_1568</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -3753,94 +3511,94 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_trip()
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 302, in &lt;module&gt;
+    main()
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 186, in main
+    rem_before_bridge = compute_remaining_need(main_city)
+                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 175, in compute_remaining_need
+    counts = count_days_per_city(presence_timeline_partial, cities)
+             ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 31, in count_days_per_city
+    counts[c] += 1
+    ~~~~~~^^^
+KeyError: None</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>trip_planning_example_125</t>
+          <t>trip_planning_example_339</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>1</v>
       </c>
       <c r="C71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 16, in &lt;module&gt;
-    result = find_itinerary(total_days, city_durations, direct_flight_pairs, friend_city, meet_window)
-             ^^^^^^^^^^^^^^
-NameError: name 'find_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Warsaw"}, {"day_range": "Day 2-8", "place": "Budapest"}, {"day_range": "Day 8-11", "place": "Paris"}, {"day_range": "Day 11-17", "place": "Riga"}]}</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>trip_planning_example_993</t>
+          <t>trip_planning_example_125</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>1</v>
       </c>
       <c r="C72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = find_itinerary()
-             ^^^^^^^^^^^^^^
-NameError: name 'find_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-6", "place": "Stuttgart"}, {"day_range": "Day 6-9", "place": "Manchester"}, {"day_range": "Day 9-15", "place": "Seville"}]}</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>trip_planning_example_996</t>
+          <t>trip_planning_example_993</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>1</v>
       </c>
       <c r="C73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E73" t="b">
@@ -3851,126 +3609,112 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "London"}, {"day_range": "Day 2-3", "place": "Amsterdam"}, {"day_range": "Day 3-7", "place": "Vilnius"}, {"day_range": "Day 7-9", "place": "Frankfurt"}, {"day_range": "Day 9-12", "place": "Bucharest"}, {"day_range": "Day 12-13", "place": "Riga"}, {"day_range": "Day 13-15", "place": "Stockholm"}]}</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>trip_planning_example_372</t>
+          <t>trip_planning_example_996</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>1</v>
       </c>
       <c r="C74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Mykonos"}, {"day_range": "Day 3-7", "place": "Zurich"}, {"day_range": "Day 7-9", "place": "Prague"}, {"day_range": "Day 9-13", "place": "Valencia"}, {"day_range": "Day 13-17", "place": "Bucharest"}, {"day_range": "Day 17-21", "place": "Riga"}, {"day_range": "Day 21-22", "place": "Nice"}]}</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>trip_planning_example_564</t>
+          <t>trip_planning_example_372</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>1</v>
       </c>
       <c r="C75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Madrid"}, {"day_range": "Day 4-5", "place": "Seville"}, {"day_range": "Day 5-7", "place": "Porto"}, {"day_range": "Day 7-13", "place": "Stuttgart"}]}</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>trip_planning_example_1167</t>
+          <t>trip_planning_example_564</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>1</v>
       </c>
       <c r="C76" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2
-    Mykonos and Naples,
-IndentationError: unexpected indent</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Seville"}, {"day_range": "Day 4-6", "place": "Rome"}, {"day_range": "Day 6-7", "place": "Istanbul"}, {"day_range": "Day 7-13", "place": "Naples"}, {"day_range": "Day 13-16", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>trip_planning_example_895</t>
+          <t>trip_planning_example_1167</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>1</v>
       </c>
       <c r="C77" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E77" t="b">
@@ -3981,161 +3725,141 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Mykonos"}, {"day_range": "Day 4-7", "place": "Naples"}, {"day_range": "Day 7-9", "place": "Istanbul"}, {"day_range": "Day 9-11", "place": "Venice"}, {"day_range": "Day 11-15", "place": "Dublin"}, {"day_range": "Day 15-16", "place": "Brussels"}, {"day_range": "Day 16-18", "place": "Frankfurt"}, {"day_range": "Day 18-21", "place": "Krakow"}]}</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>trip_planning_example_188</t>
+          <t>trip_planning_example_895</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>1</v>
       </c>
       <c r="C78" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Brussels"}, {"day_range": "Day 2-5", "place": "Lisbon"}, {"day_range": "Day 5-7", "place": "Venice"}, {"day_range": "Day 7-11", "place": "Madrid"}, {"day_range": "Day 11-13", "place": "Santorini"}, {"day_range": "Day 13-15", "place": "London"}, {"day_range": "Day 15-17", "place": "Reykjavik"}]}</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>trip_planning_example_1094</t>
+          <t>trip_planning_example_188</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>1</v>
       </c>
       <c r="C79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Brussels"}, {"day_range": "Day 2-8", "place": "Barcelona"}, {"day_range": "Day 8-12", "place": "Split"}]}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>trip_planning_example_1147</t>
+          <t>trip_planning_example_1094</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>1</v>
       </c>
       <c r="C80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 47, in &lt;module&gt;
-    result = compute_itinerary(total_days, durations, presence_windows, flights_list)
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Paris"}, {"day_range": "Day 2-4", "place": "Krakow"}, {"day_range": "Day 4-7", "place": "Vienna"}, {"day_range": "Day 7-10", "place": "Riga"}, {"day_range": "Day 10-11", "place": "Hamburg"}, {"day_range": "Day 11-12", "place": "Barcelona"}, {"day_range": "Day 12-15", "place": "Edinburgh"}, {"day_range": "Day 15-16", "place": "Stockholm"}]}</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>trip_planning_example_1450</t>
+          <t>trip_planning_example_1147</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>1</v>
       </c>
       <c r="C81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Istanbul"}, {"day_range": "Day 5-7", "place": "Brussels"}, {"day_range": "Day 7-10", "place": "Milan"}, {"day_range": "Day 10-13", "place": "Split"}, {"day_range": "Day 13-15", "place": "Helsinki"}, {"day_range": "Day 15-16", "place": "Dubrovnik"}, {"day_range": "Day 16-18", "place": "Frankfurt"}, {"day_range": "Day 18-22", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>trip_planning_example_1097</t>
+          <t>trip_planning_example_1450</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>1</v>
       </c>
       <c r="C82" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E82" t="b">
@@ -4146,183 +3870,159 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Florence"}, {"day_range": "Day 2-5", "place": "Frankfurt"}, {"day_range": "Day 5-9", "place": "Krakow"}, {"day_range": "Day 9-13", "place": "Munich"}, {"day_range": "Day 13-17", "place": "Hamburg"}, {"day_range": "Day 17-21", "place": "Oslo"}, {"day_range": "Day 21-25", "place": "Vilnius"}, {"day_range": "Day 25-29", "place": "Istanbul"}, {"day_range": "Day 29-31", "place": "Stockholm"}, {"day_range": "Day 31-32", "place": "Santorini"}]}</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>trip_planning_example_361</t>
+          <t>trip_planning_example_1097</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>1</v>
       </c>
       <c r="C83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Warsaw"}, {"day_range": "Day 4-5", "place": "Riga"}, {"day_range": "Day 5-7", "place": "Oslo"}, {"day_range": "Day 7-8", "place": "Dubrovnik"}, {"day_range": "Day 8-9", "place": "Madrid"}, {"day_range": "Day 9-13", "place": "Lyon"}, {"day_range": "Day 13-15", "place": "London"}, {"day_range": "Day 15-18", "place": "Reykjavik"}]}</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>trip_planning_example_587</t>
+          <t>trip_planning_example_361</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>1</v>
       </c>
       <c r="C84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 26, in &lt;module&gt;
-    result = generate_itinerary(
-             ^^^^^^^^^^^^^^^^^^
-NameError: name 'generate_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Madrid"}, {"day_range": "Day 7-9", "place": "Seville"}, {"day_range": "Day 9-14", "place": "Paris"}, {"day_range": "Day 14-15", "place": "Bucharest"}]}</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>trip_planning_example_656</t>
+          <t>trip_planning_example_587</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>1</v>
       </c>
       <c r="C85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_itinerary()
-             ^^^^^^^^^^^^^^
-NameError: name 'plan_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Manchester"}, {"day_range": "Day 3-9", "place": "Venice"}, {"day_range": "Day 9-10", "place": "Lyon"}, {"day_range": "Day 10-16", "place": "Istanbul"}, {"day_range": "Day 16-21", "place": "Krakow"}]}</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>trip_planning_example_824</t>
+          <t>trip_planning_example_656</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>1</v>
       </c>
       <c r="C86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Bucharest"}, {"day_range": "Day 5-8", "place": "Istanbul"}, {"day_range": "Day 8-9", "place": "Oslo"}, {"day_range": "Day 9-13", "place": "Reykjavik"}, {"day_range": "Day 13-15", "place": "Stuttgart"}, {"day_range": "Day 15-19", "place": "Edinburgh"}]}</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>trip_planning_example_1434</t>
+          <t>trip_planning_example_824</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>1</v>
       </c>
       <c r="C87" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Berlin"}, {"day_range": "Day 5-7", "place": "Split"}, {"day_range": "Day 7-11", "place": "Lyon"}, {"day_range": "Day 11-13", "place": "Lisbon"}, {"day_range": "Day 13-15", "place": "Bucharest"}, {"day_range": "Day 15-19", "place": "Riga"}, {"day_range": "Day 19-22", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>trip_planning_example_1066</t>
+          <t>trip_planning_example_1434</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -4345,61 +4045,61 @@
       <c r="G88" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 268, in &lt;module&gt;
     main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 251, in main
+    result = compute_itinerary(
+             ^^^^^^^^^^^^^^^^^^
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 198, in compute_itinerary
+    raise RuntimeError("No feasible itinerary found under given constraints.")
+RuntimeError: No feasible itinerary found under given constraints.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>trip_planning_example_995</t>
+          <t>trip_planning_example_1066</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>1</v>
       </c>
       <c r="C89" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Stuttgart"}, {"day_range": "Day 4-6", "place": "Split"}, {"day_range": "Day 6-10", "place": "Helsinki"}, {"day_range": "Day 10-13", "place": "Brussels"}, {"day_range": "Day 13-15", "place": "Bucharest"}, {"day_range": "Day 15-19", "place": "London"}, {"day_range": "Day 19-20", "place": "Mykonos"}, {"day_range": "Day 20-21", "place": "Madrid"}]}</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>trip_planning_example_875</t>
+          <t>trip_planning_example_995</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>1</v>
       </c>
       <c r="C90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Wrong plan</t>
         </is>
       </c>
       <c r="E90" t="b">
@@ -4410,249 +4110,217 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Barcelona"}, {"day_range": "Day 3-4", "place": "Oslo"}, {"day_range": "Day 4-7", "place": "Venice"}, {"day_range": "Day 7-9", "place": "Brussels"}, {"day_range": "Day 9-11", "place": "Copenhagen"}, {"day_range": "Day 11-13", "place": "Stuttgart"}, {"day_range": "Day 13-16", "place": "Split"}]}</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>trip_planning_example_1549</t>
+          <t>trip_planning_example_875</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>1</v>
       </c>
       <c r="C91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = build_itinerary()
-             ^^^^^^^^^^^^^^^
-NameError: name 'build_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Venice"}, {"day_range": "Day 5-8", "place": "Edinburgh"}, {"day_range": "Day 8-11", "place": "Krakow"}, {"day_range": "Day 11-13", "place": "Stuttgart"}, {"day_range": "Day 13-14", "place": "Split"}, {"day_range": "Day 14-17", "place": "Athens"}, {"day_range": "Day 17-20", "place": "Mykonos"}]}</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>trip_planning_example_50</t>
+          <t>trip_planning_example_1549</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>1</v>
       </c>
       <c r="C92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 16, in &lt;module&gt;
-    result = plan_trip(total_days, city_days, direct_flights)
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Lisbon"}, {"day_range": "Day 5-8", "place": "Riga"}, {"day_range": "Day 8-9", "place": "Stockholm"}, {"day_range": "Day 9-13", "place": "Santorini"}, {"day_range": "Day 13-17", "place": "Naples"}, {"day_range": "Day 17-18", "place": "Warsaw"}, {"day_range": "Day 18-20", "place": "Tallinn"}, {"day_range": "Day 20-24", "place": "Prague"}, {"day_range": "Day 24-26", "place": "Milan"}, {"day_range": "Day 26-28", "place": "Porto"}]}</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>trip_planning_example_1324</t>
+          <t>trip_planning_example_50</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>1</v>
       </c>
       <c r="C93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Vilnius"}, {"day_range": "Day 4-6", "place": "Munich"}, {"day_range": "Day 6-12", "place": "Mykonos"}]}</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>trip_planning_example_580</t>
+          <t>trip_planning_example_1324</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>1</v>
       </c>
       <c r="C94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F94" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = plan_trip()
-             ^^^^^^^^^
-NameError: name 'plan_trip' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Lyon"}, {"day_range": "Day 4-7", "place": "Venice"}, {"day_range": "Day 7-10", "place": "Copenhagen"}, {"day_range": "Day 10-12", "place": "Barcelona"}, {"day_range": "Day 12-15", "place": "Reykjavik"}, {"day_range": "Day 15-16", "place": "Athens"}, {"day_range": "Day 16-20", "place": "Dubrovnik"}, {"day_range": "Day 20-22", "place": "Munich"}, {"day_range": "Day 22-26", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>trip_planning_example_664</t>
+          <t>trip_planning_example_580</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>1</v>
       </c>
       <c r="C95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = {"itinerary": compute_itinerary()}
-                           ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-7", "place": "Geneva"}, {"day_range": "Day 7-13", "place": "Porto"}, {"day_range": "Day 13-18", "place": "Paris"}, {"day_range": "Day 18-19", "place": "Reykjavik"}, {"day_range": "Day 19-23", "place": "Oslo"}]}</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>trip_planning_example_1392</t>
+          <t>trip_planning_example_664</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>1</v>
       </c>
       <c r="C96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F96" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+          <t>{"itinerary": [{"day_range": "Day 1-4", "place": "Bucharest"}, {"day_range": "Day 4-8", "place": "Munich"}, {"day_range": "Day 8-12", "place": "Seville"}, {"day_range": "Day 12-13", "place": "Milan"}, {"day_range": "Day 13-17", "place": "Stockholm"}, {"day_range": "Day 17-18", "place": "Tallinn"}]}</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>trip_planning_example_1161</t>
+          <t>trip_planning_example_1392</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>1</v>
       </c>
       <c r="C97" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Split"}, {"day_range": "Day 5-6", "place": "Barcelona"}, {"day_range": "Day 6-10", "place": "Venice"}, {"day_range": "Day 10-11", "place": "Stuttgart"}, {"day_range": "Day 11-14", "place": "Porto"}, {"day_range": "Day 14-18", "place": "Valencia"}, {"day_range": "Day 18-20", "place": "Naples"}, {"day_range": "Day 20-23", "place": "Amsterdam"}, {"day_range": "Day 23-24", "place": "Nice"}]}</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>trip_planning_example_464</t>
+          <t>trip_planning_example_1161</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -4675,76 +4343,99 @@
       <c r="G98" t="inlineStr">
         <is>
           <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    main()
-    ^^^^
-NameError: name 'main' is not defined. Did you mean: 'min'?</t>
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 180, in &lt;module&gt;
+    result = compute_itinerary()
+             ^^^^^^^^^^^^^^^^^^^
+  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-24 21:24:11.py", line 142, in compute_itinerary
+    raise ValueError(f"Constraint violation: {city} has {city_days.get(city, 0)} days, requires {req}")
+ValueError: Constraint violation: Helsinki has 3 days, requires 2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>trip_planning_example_87</t>
+          <t>trip_planning_example_464</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>1</v>
       </c>
       <c r="C99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="E99" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F99" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+          <t>{"itinerary": [{"day_range": "Day 1-5", "place": "Naples"}, {"day_range": "Day 5-9", "place": "Dubrovnik"}, {"day_range": "Day 9-12", "place": "Frankfurt"}, {"day_range": "Day 12-16", "place": "Krakow"}, {"day_range": "Day 16-18", "place": "Oslo"}]}</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>trip_planning_example_87</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>1</v>
+      </c>
+      <c r="C100" t="b">
+        <v>0</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="E100" t="b">
+        <v>1</v>
+      </c>
+      <c r="F100" t="b">
+        <v>1</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>{"itinerary": [{"day_range": "Day 1-2", "place": "Riga"}, {"day_range": "Day 2-3", "place": "Amsterdam"}, {"day_range": "Day 3-7", "place": "Mykonos"}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>trip_planning_example_810</t>
         </is>
       </c>
-      <c r="B100" t="n">
-        <v>1</v>
-      </c>
-      <c r="C100" t="b">
-        <v>1</v>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="E100" t="b">
-        <v>0</v>
-      </c>
-      <c r="F100" t="b">
-        <v>0</v>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>Traceback (most recent call last):
-  File "/local-ssd/rma336/calendar-planning/source/generated_code_trip_2025-08-08 17:57:00.py", line 2, in &lt;module&gt;
-    result = compute_itinerary()
-             ^^^^^^^^^^^^^^^^^
-NameError: name 'compute_itinerary' is not defined</t>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" t="b">
+        <v>0</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="E101" t="b">
+        <v>1</v>
+      </c>
+      <c r="F101" t="b">
+        <v>1</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>{"itinerary": [{"day_range": "Day 1-3", "place": "Berlin"}, {"day_range": "Day 3-4", "place": "Barcelona"}, {"day_range": "Day 4-5", "place": "Lyon"}, {"day_range": "Day 5-9", "place": "Nice"}, {"day_range": "Day 9-13", "place": "Stockholm"}, {"day_range": "Day 13-17", "place": "Athens"}, {"day_range": "Day 17-20", "place": "Vilnius"}]}</t>
         </is>
       </c>
     </row>

</xml_diff>